<commit_message>
Consolidated into maia-clara, removed content.
Removed content from files in this repository.
</commit_message>
<xml_diff>
--- a/wishlist_maia.xlsx
+++ b/wishlist_maia.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cfn7021\Downloads\wishlist\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59519CC7-9A7E-4FD9-8DC8-77FFFEAF63F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5CE5DEB-00A5-4957-AA7C-00CCF8D4E32E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38400" yWindow="0" windowWidth="19200" windowHeight="23400" xr2:uid="{FE4DC328-739C-48AF-B2EF-9BDF321350CE}"/>
+    <workbookView xWindow="4290" yWindow="615" windowWidth="29010" windowHeight="23385" xr2:uid="{FE4DC328-739C-48AF-B2EF-9BDF321350CE}"/>
   </bookViews>
   <sheets>
-    <sheet name="Clara" sheetId="1" r:id="rId1"/>
+    <sheet name="Maia" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Clara!$A$1:$E$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Maia!$A$1:$E$24</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>Image</t>
   </si>
@@ -53,19 +53,7 @@
     <t>Name</t>
   </si>
   <si>
-    <t>https://www.amazon.de/dp/3741524727?psc=1&amp;ref_=cm_sw_r_cp_ud_ct_WRC2J9TPX505376KF519</t>
-  </si>
-  <si>
-    <t>https://m.media-amazon.com/images/I/71IQvmivQSL.jpg</t>
-  </si>
-  <si>
-    <t>Magic Water Colouring</t>
-  </si>
-  <si>
-    <t>9 EUR</t>
-  </si>
-  <si>
-    <t>Reserved / bought</t>
+    <t>SKIP (skip: hide from display) / Y (reserved: show faded out) / GAP (formatting gap)</t>
   </si>
 </sst>
 </file>
@@ -147,9 +135,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -187,7 +175,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -293,7 +281,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -435,7 +423,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -448,7 +436,7 @@
   <cols>
     <col min="1" max="2" width="26.140625" customWidth="1"/>
     <col min="3" max="3" width="53.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="79" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -465,21 +453,7 @@
         <v>2</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -550,10 +524,13 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D24">
     <sortCondition ref="D3:D24"/>
   </sortState>
-  <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{A46C8FBB-687F-4272-856C-B9A2E282C9A5}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{ff6dbec8-95a8-4638-9f5f-bd076536645c}" enabled="1" method="Standard" siteId="{5dbf1add-202a-4b8d-815b-bf0fb024e033}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>